<commit_message>
Cập nhật skill + plan các feature mới
- Bổ sung quy tắc vào CLAUDE.md và các skill (button, entity-history,
  info-icon-tooltip, list-page)
- Thêm plan: dong-bo-quy-tac-chung, history-action-groups,
  redmine-11058-icon-info-giai-doan-du-an, status-color-convention,
  sync-assign-catalogs
- Cập nhật STATUS.md

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hrm/.plans/meeting-create-bugfix/thong-bao-meeting.xlsx
+++ b/hrm/.plans/meeting-create-bugfix/thong-bao-meeting.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,7 +33,6 @@
       <sz val="14"/>
     </font>
     <font>
-      <i val="1"/>
       <color rgb="00666666"/>
       <sz val="10"/>
     </font>
@@ -48,17 +47,11 @@
       <sz val="11"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00006100"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="009C0006"/>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="7">
@@ -85,12 +78,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -104,35 +97,37 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00B7C3D0"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00B7C3D0"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00B7C3D0"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00B7C3D0"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -143,17 +138,14 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -520,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -538,21 +530,21 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cập nhật 11/08/2026 theo code hiện tại  |  Module Giao việc (Assign)  |  Mỗi thông báo đẩy 3 kênh: chuông web (Redis) + push mobile + bản ghi DB</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t>Cập nhật 14/08/2026 sau khi merge nhánh tpe-develop-assign vào tpe  |  Module Giao việc  |  Phần xử lý thông báo chốt giữ theo bản tpe-develop-assign: nút Lưu KHÔNG gửi cờ send_notification, BE tự so sánh dữ liệu trước/sau để báo đúng người.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="26" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Người nhận luôn là THÀNH VIÊN NỘI BỘ (tab Thành viên công ty). Thành viên khách hàng không nhận gì. Người tạo/người thao tác nằm trong danh sách thành viên nên cũng nhận.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="26" customHeight="1">
+          <t>Người nhận luôn là THÀNH VIÊN NỘI BỘ (tab Thành viên công ty) — thành viên khách hàng không nhận gì. Mỗi thông báo = 1 lần gửi, đẩy đồng thời 3 kênh (chuông realtime, push mobile, bảng notifications).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>STT</t>
@@ -584,7 +576,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="22" customHeight="1">
+    <row r="6" ht="20" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>MÀN TẠO MỚI  (POST /assign/meeting)</t>
@@ -596,11 +588,9 @@
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
     </row>
-    <row r="7" ht="62" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
@@ -624,15 +614,13 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>MeetingController::store():180 — status 0 không khớp nhánh nào</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="62" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+          <t>MeetingController::store():180 — status 0 không khớp nhánh nào trong service</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>2</v>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
@@ -651,447 +639,529 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>[Meeting]: &lt;b&gt;Tên meeting&lt;/b&gt;. Thời gian dự kiến (12/08/2026 14:00:00 - 12/08/2026 16:00:00) Địa điểm: … Hình thức: Trực tiếp</t>
+          <t>[Meeting]: &lt;b&gt;Tên meeting&lt;/b&gt;. Thời gian dự kiến (14:00 12/08/2026 - 16:00 12/08/2026) Địa điểm: … Hình thức: …</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>MeetingController::store():180 → MeetingService::sendMeetingNotification():1088</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+          <t>MeetingController::store():180 → MeetingService::sendMeetingNotification():1110</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Bấm 'Đã chốt lịch'</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Tạo meeting ở trạng thái Chốt lịch (2)</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Toàn bộ thành viên nội bộ của cuộc họp</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>[Meeting]: &lt;b&gt;Tên meeting&lt;/b&gt;. Thời gian (…) Địa điểm: … Hình thức: …</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>MeetingController::store():180 → MeetingService::sendMeetingNotification():1129</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>MÀN SỬA — NÚT CHUYỂN TRẠNG THÁI  (PUT /assign/meeting/{id})</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="5" t="n"/>
-    </row>
-    <row r="10" ht="62" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Bấm 'Lên lịch hẹn'</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Trạng thái đổi (vd 0 → 1)</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Trạng thái đổi (0 → 1). FE gửi send_notification = 1</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>Toàn bộ thành viên nội bộ của cuộc họp</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>[Meeting]: &lt;b&gt;Tên meeting&lt;/b&gt;. Thời gian dự kiến (…) Địa điểm: … Hình thức: …</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr">
-        <is>
-          <t>MeetingController::update():349 → MeetingService::sendMeetingNotification()</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="62" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>MeetingForm.vue:751 → MeetingController::update():354 → MeetingService:1110</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Bấm 'Đã chốt lịch'</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Trạng thái đổi (1 → 2)</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Trạng thái đổi (1 → 2). FE không gửi cờ → BE mặc định gửi</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>Toàn bộ thành viên nội bộ của cuộc họp</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>[Meeting]: &lt;b&gt;Tên meeting&lt;/b&gt;. Thời gian (…) Địa điểm: … Hình thức: …</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>MeetingController::update():349 → MeetingService::sendMeetingNotification():1106</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>MÀN SỬA — NÚT 'LƯU' (giữ nguyên trạng thái Lên lịch hoặc Chốt lịch)</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-    </row>
-    <row r="13" ht="62" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>MeetingForm.vue:756 → MeetingController::update():354 → MeetingService:1129</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>MÀN SỬA — NÚT 'LƯU' (giữ nguyên trạng thái Lên lịch hoặc Chốt lịch) — BE tự quyết báo cho ai</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Bấm 'Lưu'</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>KHÔNG đổi giờ, KHÔNG thêm/bớt người
-(chỉ sửa ghi chú, biên bản, điểm danh, dự án…)</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
+(chỉ sửa ghi chú, biên bản, dự án…)</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
         <is>
           <t>Không ai</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>— Không báo cho ai</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>MeetingService::notifyMeetingChanges() — thoát sớm khi không có thay đổi</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="62" customHeight="1">
-      <c r="A14" s="6" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
+        <is>
+          <t>MeetingService::notifyMeetingChanges():1157 — thoát sớm khi không có thay đổi đáng báo</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Bấm 'Lưu'</t>
         </is>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>CÓ đổi thời gian họp
 (start_date hoặc end_date)</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>Thành viên nội bộ đang ở trong meeting
-(KHÔNG gồm người vừa được thêm ở cùng lần lưu)</t>
-        </is>
-      </c>
-      <c r="E14" s="7" t="inlineStr">
+(KHÔNG gồm người vừa được thêm)</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>[MET] Thay đổi lịch: &lt;b&gt;Tên meeting&lt;/b&gt;. Thời gian mới: 14:00 - 16:00 12/08/2026</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>MeetingService::notifyMeetingChanges() — nhóm 'kept'</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="62" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Bấm 'Lưu'</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>CÓ thêm người nội bộ mới</t>
         </is>
       </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Chỉ người vừa được thêm</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>[MET] Cập nhật: &lt;b&gt;Tên meeting&lt;/b&gt;. Bạn được thêm vào cuộc họp. Thời gian: 14:00 - 16:00 12/08/2026</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>MeetingService::notifyMeetingChanges() — nhóm 'added'</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="62" customHeight="1">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Bấm 'Lưu'</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>CÓ bỏ người nội bộ khỏi cuộc họp</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>Chỉ người bị đưa ra khỏi cuộc họp</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>[MET] Cập nhật: &lt;b&gt;Tên meeting&lt;/b&gt;. Bạn đã được đưa ra khỏi cuộc họp.</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>MeetingService::notifyMeetingChanges() — nhóm 'removed'</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="62" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Bấm 'Lưu'</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C18" s="7" t="inlineStr">
         <is>
           <t>VỪA đổi giờ VỪA thêm/bớt người</t>
         </is>
       </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Mỗi người đúng 1 thông báo:
 • người cũ ở lại → noti đổi lịch
 • người mới → noti được thêm
-• người bị bỏ → noti đưa ra khỏi họp</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>Kết hợp 3 nội dung ở mục 6, 7, 8 — người mới KHÔNG nhận thêm noti đổi lịch</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
+• người bị bỏ → noti bị đưa ra</t>
+        </is>
+      </c>
+      <c r="E18" s="7" t="inlineStr">
+        <is>
+          <t>Kết hợp 3 nội dung ở mục 7, 8, 9 — người mới KHÔNG nhận thêm noti đổi lịch</t>
+        </is>
+      </c>
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>MeetingService::notifyMeetingChanges()</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="62" customHeight="1">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Bấm 'Lưu' + đổi giờ khi ĐÃ CHỐT LỊCH</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>Popup xác nhận đổi thời gian → Đồng ý</t>
         </is>
       </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="D19" s="9" t="inlineStr">
         <is>
           <t>Thành viên nội bộ đang ở trong meeting</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>Giống mục 6 (nội dung [MET] Thay đổi lịch với giờ mới)</t>
-        </is>
-      </c>
-      <c r="F18" s="7" t="inlineStr">
-        <is>
-          <t>MeetingForm.vue::confirmTimeChange() → cùng luồng mục 6</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>Giống mục 7 ([MET] Thay đổi lịch, kèm giờ mới)</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>MeetingForm.vue::confirmTimeChange():948 → cùng luồng mục 7</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>CÁC THAO TÁC KHÁC</t>
         </is>
       </c>
-      <c r="B19" s="5" t="n"/>
-      <c r="C19" s="5" t="n"/>
-      <c r="D19" s="5" t="n"/>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="n"/>
-    </row>
-    <row r="20" ht="62" customHeight="1">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="5" t="n"/>
+      <c r="C20" s="5" t="n"/>
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="5" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Bấm 'Hoàn thành' (chốt biên bản)</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>Trạng thái 2 → 3</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>Không ai</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
         <is>
           <t>— BE không có nhánh xử lý status 3</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>MeetingService::sendMeetingNotification() chỉ xử lý status 1 và 2</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="62" customHeight="1">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="B21" s="7" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Bấm 'Huỷ' → nhập lý do → xác nhận</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>Trạng thái → 4 (Huỷ)</t>
         </is>
       </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Toàn bộ thành viên nội bộ của cuộc họp</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>&lt;b&gt;Tên meeting&lt;/b&gt; đã bị &lt;b&gt;Người huỷ&lt;/b&gt; huỷ. Lý do: …</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F22" s="7" t="inlineStr">
         <is>
           <t>MeetingController::changeStatus():225 → hàm private sendMeetingNotification():543</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="62" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B22" s="7" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Bấm 'Xoá' meeting nháp</t>
         </is>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>Chỉ xoá được khi ở trạng thái 0</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr">
+      <c r="D23" s="8" t="inlineStr">
         <is>
           <t>Không ai</t>
         </is>
       </c>
-      <c r="E22" s="7" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F22" s="7" t="inlineStr">
-        <is>
-          <t>MeetingController::destroy()</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="62" customHeight="1">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>Nhắc trước giờ họp (reminder)</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="F23" s="7" t="inlineStr">
+        <is>
+          <t>MeetingController::destroy() — không gọi hàm thông báo nào</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>TỰ ĐỘNG (cron 15 phút/lần — assign:meeting-report-deadline, Redmine #11014)</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n"/>
+      <c r="C24" s="5" t="n"/>
+      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="5" t="n"/>
+      <c r="F24" s="5" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Nhắc nhập biên bản trước hạn tự huỷ</t>
+        </is>
+      </c>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>Meeting đã họp xong, chưa nhập biên bản, gần tới hạn</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>CHỈ người tạo meeting (created_by)</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>[MET] Nhắc báo cáo: &lt;b&gt;Tên meeting&lt;/b&gt;. Chưa có biên bản, sẽ tự hủy lúc 17:00 15/08.</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>MeetingService::notifyReportReminder():1207 · app/Console/Kernel.php:62</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>Tự động huỷ cuộc họp quá hạn nhập biên bản</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>Quá hạn nhập biên bản</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>Toàn bộ thành viên nội bộ + người tạo</t>
+        </is>
+      </c>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>[MET] Hủy: &lt;b&gt;Tên meeting&lt;/b&gt;. Quá hạn nhập biên bản.</t>
+        </is>
+      </c>
+      <c r="F26" s="7" t="inlineStr">
+        <is>
+          <t>MeetingService::autoCancelOverdueMeeting():1242</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Nhắc trước GIỜ HỌP (reminder lịch)</t>
+        </is>
+      </c>
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr">
+      <c r="D27" s="8" t="inlineStr">
         <is>
           <t>Không ai</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
-        <is>
-          <t>— Hệ thống KHÔNG có cron/job nhắc lịch trước giờ họp</t>
-        </is>
-      </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>Không có schedule liên quan meeting trong app/Console/Kernel.php</t>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>— Hệ thống KHÔNG có cron nhắc trước giờ họp (chỉ có cron nhắc biên bản ở mục 15)</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr">
+        <is>
+          <t>Không có schedule nào khác liên quan meeting trong app/Console/Kernel.php</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A19:F19"/>
+  <mergeCells count="8">
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A6:F6"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A20:F20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1103,12 +1173,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="105" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -1141,11 +1211,9 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+    <row r="4">
+      <c r="A4" s="6" t="n">
+        <v>1</v>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
@@ -1159,15 +1227,13 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Lấy từ bảng meeting_employees (type = 1, có employee_id) → employee_info_id. Thành viên khách hàng (type = 2) không nhận thông báo, không email, không SMS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="60" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+          <t>Lấy từ bảng meeting_employees (có employee_id) → employee_info_id. Thành viên khách hàng không nhận email/SMS/noti. Người tạo meeting được FE tự thêm vào danh sách nên cũng nhận.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>2</v>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
@@ -1181,188 +1247,214 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>EmployeeInfoService::sendNotification() bắn đồng thời: Redis publish (chuông web realtime), job SendNotification (push mobile), và ghi bảng notifications (danh sách chuông).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+          <t>EmployeeInfoService::sendNotification() bắn đồng thời: Redis publish (chuông realtime), job push mobile, ghi bảng notifications. Đây là 1 thông báo — không tính là lặp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>3</v>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Chuẩn nội dung mới</t>
+          <t>1 hành động = 1 thông báo (KHÔNG lặp)</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>ÁP DỤNG TỪ 11/08/2026</t>
+          <t>ĐÃ SỬA — còn đúng sau merge</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Các thông báo mới theo template [PREFIX] {Nhóm hành động}: {Tên đối tượng}. {Ghi chú} — prefix [MET], tên in đậm cắt còn 50 ký tự, tổng nội dung ≤ 120 ký tự (cắt ghi chú trước). Xem .claude/skills/notification-convention/SKILL.md</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+          <t>Lỗi cũ: update() gọi CẢ MeetingService::sendMeetingNotification VÀ hàm private của controller → 1 hành động ra 2 noti khác nội dung. Hiện update() chỉ gọi service đúng 1 lần trong if ($shouldNotify); hàm private chỉ còn phục vụ luồng Huỷ. Đã rà lại toàn bộ caller ngày 14/08/2026: không còn điểm nào bắn trùng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n">
+        <v>4</v>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
+          <t>Trùng người nhận trong 1 lần gửi</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>QUY TẮC</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Danh sách employee_info_id được array_unique trước khi gửi (kể cả luồng cron gộp thành viên + người tạo) → 1 người chỉ nhận 1 bản.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
           <t>Deep-link</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>QUY TẮC</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Mọi thông báo đều có url = /assign/meeting/{id}/show (kèm ID), type = 'meeting'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="inlineStr">
-        <is>
-          <t>1 hành động = 1 thông báo</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>ĐÃ SỬA 11/08/2026</t>
-        </is>
-      </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Trước đây hàm update() gọi cả MeetingService::sendMeetingNotification lẫn hàm private cùng tên của controller → mỗi lần bấm Lên lịch/Chốt lịch ở màn Sửa bắn 2 noti nội dung khác nhau. Nay chỉ còn 1 nguồn; hàm private chỉ phục vụ luồng Huỷ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
+          <t>Mọi thông báo đều có url = /assign/meeting/{id}/show (kèm ID) và type = 'meeting'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n">
+        <v>6</v>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
+          <t>Cron nhắc biên bản không gửi lặp</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>QUY TẮC</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Cron chạy 15 phút/lần nhưng notifyReportReminder() kiểm tra cờ report_deadline_notified_at → mỗi meeting chỉ nhắc 1 lần. Job tự huỷ cũng chỉ vào được khi meeting còn đang chờ biên bản, huỷ xong status = 4 nên lần sau bỏ qua.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
           <t>Gửi sau khi commit</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
-        <is>
-          <t>ĐÃ SỬA ở update()
-CÒN ở store()</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>Ở update() thông báo đã được gửi sau DB::commit(). Ở store() (tạo mới) lời gọi vẫn nằm trong transaction (MeetingController:180 trước :182) → nếu rollback vẫn bắn noti trỏ tới meeting không tồn tại.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="60" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>ĐÃ SỬA ở update() — CÒN ở store()</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>update() gửi sau DB::commit(). store() vẫn gửi ở dòng 180, trước commit dòng 182 → nếu rollback thì noti/push đã bắn nhưng meeting không tồn tại (link 404). ĐỀ XUẤT: chuyển xuống sau commit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Nút 'Lưu' báo đúng người bị ảnh hưởng</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>GIỮ THEO tpe-develop-assign</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>FE KHÔNG gửi cờ send_notification ở nút 'Lưu'; BE so sánh snapshot trước/sau khi sync để quyết định: đổi giờ → báo toàn bộ thành viên đang ở trong meeting; thêm/bớt người → chỉ báo người liên quan; không đổi gì → không báo ai. Hành vi này được chốt khi merge ngày 14/08/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Người mới thêm chỉ nhận 1 thông báo</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>QUY TẮC</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Khi vừa đổi giờ vừa thêm người: người mới chỉ nhận noti 'Bạn được thêm vào cuộc họp' (đã kèm giờ), KHÔNG nhận thêm noti đổi lịch — nhóm 'kept' chỉ gồm người có mặt ở cả trước và sau.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Người thao tác tự nhận thông báo của chính mình</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C13" s="12" t="inlineStr">
         <is>
           <t>CÒN TỒN ĐỌNG</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>Danh sách nhận không loại trừ người đang bấm nút. Người tự chốt lịch / tự đổi giờ vẫn nhận noti. Sửa được bằng cách loại auth()-&gt;user() khỏi danh sách trước khi gửi — chưa làm vì chưa có yêu cầu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="60" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>Nội dung nhánh đổi trạng thái chưa theo chuẩn mới</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>Danh sách nhận không loại trừ người đang bấm nút — người tự chốt lịch vẫn nhận noti do chính mình gây ra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Nội dung chưa thống nhất template</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>CÒN TỒN ĐỌNG</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>Nút Lên lịch hẹn / Đã chốt lịch vẫn dùng câu cũ '[Meeting]: &lt;tên&gt;. Thời gian (…)' thay vì '[MET] {Nhóm hành động}: …'. Chưa đổi vì sẽ thay câu chữ người dùng đang quen — cần chốt trước khi chuẩn hoá.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="60" customHeight="1">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>9</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Không có nhắc lịch tự động</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>HIỆN TRẠNG</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>Không có cron/job nhắc trước giờ họp. Muốn có phải làm mới (schedule + điều kiện thời điểm nhắc).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Cờ send_notification</t>
-        </is>
-      </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>HIỆN TRẠNG</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>BE vẫn nhận field send_notification (mặc định true) để tắt thông báo khi cần. FE màn meeting không còn gửi cờ này nữa — BE tự so sánh dữ liệu trước/sau để quyết định báo cho ai.</t>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>Nút Lên lịch / Chốt lịch và luồng Huỷ vẫn dùng câu cũ ('[Meeting]: …', '&lt;b&gt;Tên&lt;/b&gt; đã bị … huỷ'); còn nút 'Lưu' và 2 luồng cron đã theo template chuẩn [MET] {Nhóm hành động}: &lt;b&gt;{Tên ≤50}&lt;/b&gt;. {Ghi chú} (.claude/skills/notification-convention). Ghi chú bị cắt nếu tổng vượt 120 ký tự.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Hoàn thành cuộc họp không có thông báo</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>CÒN TỒN ĐỌNG</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>Service không có nhánh status 3 → chốt biên bản xong không ai được báo. Cần xác nhận đúng nghiệp vụ hay bỏ sót.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1373,7 +1465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1405,7 +1497,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="52" customHeight="1">
+    <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>MeetingService::sendMeetingNotification()</t>
@@ -1413,152 +1505,189 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Modules/Assign/Services/MeetingService.php:1072</t>
+          <t>hrm-api/Modules/Assign/Services/MeetingService.php:1094</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Báo TOÀN BỘ thành viên nội bộ khi chuyển trạng thái sang Lên lịch (1) hoặc Chốt lịch (2). Dùng ở cả tạo mới và sửa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>MeetingService::notifyMeetingChanges()  ★ MỚI</t>
+          <t>Nguồn chính: báo TOÀN BỘ thành viên nội bộ khi status = 1 (Lên lịch) hoặc 2 (Chốt lịch). Status khác → không gửi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>MeetingController::sendMeetingNotification() (private)</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Modules/Assign/Services/MeetingService.php:1126</t>
+          <t>hrm-api/Modules/Assign/Http/Controllers/Api/V1/MeetingController.php:543</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Bấm 'Lưu' mà không đổi trạng thái: so sánh snapshot trước/sau → chia 3 nhóm kept (đổi giờ) / added (được thêm) / removed (bị bỏ) và chỉ báo đúng người liên quan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>buildMeetingNotificationContent()  ★ MỚI</t>
+          <t>CHỈ còn phục vụ luồng Huỷ (status 4), gọi từ changeStatus().</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>MeetingController::store()</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Modules/Assign/Services/MeetingService.php (private)</t>
+          <t>hrm-api/Modules/Assign/Http/Controllers/Api/V1/MeetingController.php:180</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Dựng chuỗi [MET] {Nhóm hành động}: &lt;b&gt;{Tên ≤50}&lt;/b&gt;. {Ghi chú}; tổng ≤ 120 ký tự, cắt ghi chú trước.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>formatMeetingTimeRange() / isSameDateTime()  ★ MỚI</t>
+          <t>Tạo mới — gọi service 1 lần, KHÔNG đọc cờ send_notification. Lưu ý: gửi trước DB::commit().</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>MeetingController::update()</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Modules/Assign/Services/MeetingService.php (private)</t>
+          <t>hrm-api/Modules/Assign/Http/Controllers/Api/V1/MeetingController.php:349-356</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Định dạng khoảng giờ họp ('14:00 - 16:00 12/08/2026') và so sánh 2 mốc thời gian bằng Carbon::parse để không lệch khi FE gửi 'H:i' còn DB lưu 'H:i:s'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="52" customHeight="1">
+          <t>Chụp snapshot start_date / end_date / company_members TRƯỚC khi sync; sau DB::commit() gửi đúng 1 lần: đổi trạng thái → sendMeetingNotification(), giữ nguyên trạng thái → notifyMeetingChanges().</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>MeetingController::update()</t>
+          <t>MeetingService::notifyMeetingChanges()</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>Modules/Assign/Http/Controllers/Api/V1/MeetingController.php:274-355</t>
+          <t>hrm-api/Modules/Assign/Services/MeetingService.php:1157</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>Chụp snapshot start_date/end_date/company_members TRƯỚC khi sync (syncCompanyMembers xoá sạch rồi tạo lại), sau DB::commit() mới quyết định: đổi trạng thái → báo tất cả; giữ nguyên trạng thái → notifyMeetingChanges().</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="52" customHeight="1">
+          <t>Bấm 'Lưu' mà KHÔNG đổi trạng thái: so sánh snapshot giờ họp / danh sách thành viên trước-sau để báo đúng người (kept / added / removed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>MeetingController::sendMeetingNotification() (private)</t>
+          <t>buildMeetingNotificationContent() / formatMeetingTimeRange() / isSameDateTime()</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>Modules/Assign/Http/Controllers/Api/V1/MeetingController.php:543</t>
+          <t>hrm-api/Modules/Assign/Services/MeetingService.php (private)</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Nay CHỈ còn phục vụ luồng Huỷ (status 4) gọi từ changeStatus().</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="52" customHeight="1">
+          <t>Dựng chuỗi [MET] {Nhóm hành động}: &lt;b&gt;{Tên ≤50}&lt;/b&gt;. {Ghi chú}; format khoảng giờ họp và so sánh mốc thời gian.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
+          <t>MeetingService::notifyReportReminder() / autoCancelOverdueMeeting()</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>hrm-api/Modules/Assign/Services/MeetingService.php:1207 / :1242</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Hai luồng cron biên bản (Redmine #11014). Chạy CLI không có auth() nên lấy người tạo meeting làm người gửi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
           <t>EmployeeInfoService::sendNotification() / sendToAllNotification()</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
-        <is>
-          <t>Modules/Timesheet/Services/EmployeeInfoService.php:466 / :511</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Helper dùng chung của hệ thống — bắn 3 kênh cho từng employee_info_id.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="52" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>MeetingForm.vue::handleSave()</t>
-        </is>
-      </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>hrm-client/pages/assign/meeting/components/MeetingForm.vue:766-783</t>
+          <t>hrm-api/Modules/Timesheet/Services/EmployeeInfoService.php:466 / :511</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Nút 'Lưu': không gửi cờ send_notification nữa, để BE tự quyết. Đổi giờ khi đã chốt lịch vẫn qua popup xác nhận.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="52" customHeight="1">
+          <t>Helper dùng chung — bắn 3 kênh cho từng employee_info_id.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
+          <t>MeetingForm.vue::handleSave() / confirmTimeChange()</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>hrm-client/pages/assign/meeting/components/MeetingForm.vue:866 / :948</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Nút 'Lưu' KHÔNG gửi cờ send_notification, để BE tự quyết; riêng đổi giờ khi đã chốt lịch phải qua popup xác nhận rồi mới save(2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Cron biên bản meeting</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>hrm-api/app/Console/Kernel.php:62</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>assign:meeting-report-deadline — chạy 15 phút/lần, timezone Asia/Ho_Chi_Minh, withoutOverlapping.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
           <t>Trạng thái meeting</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
-        <is>
-          <t>Modules/Assign/Entities/Meeting/Meeting.php:62-66</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>hrm-api/Modules/Assign/Entities/Meeting/Meeting.php</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>0 Đang tạo · 1 Lên lịch · 2 Chốt lịch · 3 Hoàn thành · 4 Huỷ</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>